<commit_message>
Fix PV gallium intensity attribution
Move the 9 kg/MW gallium factor from c-Si PV to CIGS PV in the source material requirements workbook and update the generated metals_db.csv aggregate.

Add a regression test to ensure gallium is not assigned to crystalline silicon PV and remains assigned to CIGS. Validation: conda run -n premise pytest tests/test_metals.py.
</commit_message>
<xml_diff>
--- a/premise/data/metals/SI_2_Material_requirements.xlsx
+++ b/premise/data/metals/SI_2_Material_requirements.xlsx
@@ -2398,7 +2398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -2658,15 +2658,15 @@
       </c>
       <c r="D6" s="80">
         <f t="shared" si="0"/>
-        <v>17.785666666666664</v>
+        <v>16.986969696969695</v>
       </c>
       <c r="E6" s="43">
         <f t="shared" si="1"/>
-        <v>6.085</v>
+        <v>6.17</v>
       </c>
       <c r="F6" s="43">
         <f t="shared" si="2"/>
-        <v>2.3199999999999998</v>
+        <v>2.32</v>
       </c>
       <c r="G6" s="43">
         <f t="shared" si="3"/>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="H6" s="39">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I6" s="61">
         <v>11</v>
@@ -2700,7 +2700,9 @@
       <c r="P6" s="61">
         <v>4.666666666666667</v>
       </c>
-      <c r="Q6" s="88"/>
+      <c r="Q6" s="88">
+        <v>9</v>
+      </c>
       <c r="R6" s="88">
         <v>5</v>
       </c>
@@ -18024,7 +18026,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0800-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
@@ -18226,51 +18228,6 @@
       <c r="S4" s="61"/>
       <c r="T4" s="88"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="C5" s="30">
-        <v>2020</v>
-      </c>
-      <c r="D5" s="80">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="E5" s="43">
-        <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="F5" s="43">
-        <f t="shared" si="2"/>
-        <v>9</v>
-      </c>
-      <c r="G5" s="43">
-        <f t="shared" si="3"/>
-        <v>9</v>
-      </c>
-      <c r="H5" s="39">
-        <f t="shared" si="4"/>
-        <v>1</v>
-      </c>
-      <c r="I5" s="61"/>
-      <c r="J5" s="61"/>
-      <c r="K5" s="61"/>
-      <c r="L5" s="61"/>
-      <c r="M5" s="61"/>
-      <c r="N5" s="61"/>
-      <c r="O5" s="61"/>
-      <c r="P5" s="61"/>
-      <c r="Q5" s="61"/>
-      <c r="R5" s="61"/>
-      <c r="S5" s="61">
-        <v>9</v>
-      </c>
-      <c r="T5" s="88"/>
-    </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
@@ -18607,7 +18564,7 @@
       <c r="T13" s="36"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E24:E42">
+  <sortState ref="E24:E42">
     <sortCondition ref="E24"/>
   </sortState>
   <mergeCells count="1">

</xml_diff>